<commit_message>
feat(school-forms): add individual SF9 reports and repair Excel templates
- Add adviser-only SF9 previews and editable draft downloads for Grades 4–10
- Populate learner details and published grades, including additional subject rows
- Repair SF8 and SF9 workbook packaging for Excel compatibility
- Restore advisory-class choices when switching forms and explain why SF9 cannot be combined
- Add school-form access, export, and workbook-integrity tests
</commit_message>
<xml_diff>
--- a/assets/templates/school-forms/sf8.xlsx
+++ b/assets/templates/school-forms/sf8.xlsx
@@ -4,10 +4,10 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="21840" windowHeight="8610" tabRatio="876" firstSheet="1" activeTab="0"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="21840" windowHeight="8610" tabRatio="876" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="School Form 8 (SF8)" sheetId="1" r:id="rId7"/>
+    <sheet name="School Form 8 (SF8)" sheetId="30" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'School Form 8 (SF8)'!$9:$10</definedName>
@@ -2414,7 +2414,7 @@
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -2814,7 +2814,7 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr codeName="Sheet28">
     <tabColor theme="9" tint="-0.499984740745262"/>

</xml_diff>